<commit_message>
Sub steps table added and seeder executed
</commit_message>
<xml_diff>
--- a/assets/Products.xlsx
+++ b/assets/Products.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="65">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -132,6 +133,90 @@
   </si>
   <si>
     <t xml:space="preserve">Solvent Recovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAIN_STEP_ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DYNAMIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Instructions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Clearance Checklist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Clearance Record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material List</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Clearance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulverization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraction Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blow Off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blow Off Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semi Concentration Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final Concentration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final Concentration Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drying Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drying Chart </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reconciliation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manager Signoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final Concentration &amp; TDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentration Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line clearance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spray Drying chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spray Drying Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtration Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethanol Stripout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drying chart</t>
   </si>
 </sst>
 </file>
@@ -178,12 +263,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.7999"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -263,7 +354,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -277,10 +368,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -352,6 +439,42 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -382,7 +505,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFBBE6FE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -618,8 +741,8 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="34.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="34.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="16.27"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="4" width="11.53"/>
   </cols>
   <sheetData>
@@ -635,1488 +758,2785 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C23" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C27" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C28" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="5" t="n">
+      <c r="C30" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="5" t="n">
+      <c r="C31" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="5" t="n">
+      <c r="C32" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C33" s="5" t="n">
+      <c r="C33" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="5" t="n">
+      <c r="C34" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C35" s="5" t="n">
+      <c r="C35" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C36" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C37" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="5" t="n">
+      <c r="C38" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="5" t="n">
+      <c r="C39" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C40" s="5" t="n">
+      <c r="C40" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C41" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C42" s="5" t="n">
+      <c r="C42" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C43" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="16" t="s">
+      <c r="B44" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C44" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C45" s="5" t="n">
+      <c r="C45" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="B46" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C46" s="5" t="n">
+      <c r="C46" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="5" t="n">
+      <c r="C47" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C48" s="5" t="n">
+      <c r="C48" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C49" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C50" s="5" t="n">
+      <c r="C50" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C51" s="5" t="n">
+      <c r="C51" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C52" s="5" t="n">
+      <c r="C52" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C53" s="5" t="n">
+      <c r="C53" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="n">
+      <c r="A54" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C54" s="5" t="n">
+      <c r="C54" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="n">
+      <c r="A55" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C55" s="5" t="n">
+      <c r="C55" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="5" t="n">
+      <c r="A56" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C56" s="5" t="n">
+      <c r="C56" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5" t="n">
+      <c r="A57" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C57" s="5" t="n">
+      <c r="C57" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="n">
+      <c r="A58" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C58" s="5" t="n">
+      <c r="C58" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="n">
+      <c r="A59" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C59" s="5" t="n">
+      <c r="C59" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="n">
+      <c r="A60" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C60" s="5" t="n">
+      <c r="C60" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5" t="n">
+      <c r="A61" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C61" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="n">
+      <c r="A62" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="7" t="s">
+      <c r="B62" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C62" s="5" t="n">
+      <c r="C62" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="n">
+      <c r="A63" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="16" t="s">
+      <c r="B63" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C63" s="5" t="n">
+      <c r="C63" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="n">
+      <c r="A64" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="7" t="s">
+      <c r="B64" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C64" s="5" t="n">
+      <c r="C64" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="n">
+      <c r="A65" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C65" s="5" t="n">
+      <c r="C65" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="5" t="n">
+      <c r="A66" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="16" t="s">
+      <c r="B66" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="C66" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="n">
+      <c r="A67" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C67" s="5" t="n">
+      <c r="C67" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="5" t="n">
+      <c r="A68" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="15" t="s">
+      <c r="B68" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C68" s="5" t="n">
+      <c r="C68" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="15"/>
+      <c r="B69" s="14"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="15"/>
+      <c r="B70" s="14"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="15"/>
+      <c r="B72" s="14"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="15"/>
+      <c r="B73" s="14"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="15"/>
+      <c r="B74" s="14"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="15"/>
+      <c r="B75" s="14"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="15"/>
+      <c r="B76" s="14"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="15"/>
+      <c r="B77" s="14"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="17"/>
+      <c r="B79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="17"/>
+      <c r="B80" s="16"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="17"/>
+      <c r="B81" s="16"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="17"/>
+      <c r="B82" s="16"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="17"/>
+      <c r="B83" s="16"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="17"/>
+      <c r="B84" s="16"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="17"/>
+      <c r="B85" s="16"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B86" s="17"/>
+      <c r="B86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="17"/>
+      <c r="B87" s="16"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B88" s="17"/>
+      <c r="B88" s="16"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B89" s="17"/>
+      <c r="B89" s="16"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B90" s="17"/>
+      <c r="B90" s="16"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B91" s="17"/>
+      <c r="B91" s="16"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B92" s="17"/>
+      <c r="B92" s="16"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B93" s="17"/>
+      <c r="B93" s="16"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B94" s="17"/>
+      <c r="B94" s="16"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B95" s="17"/>
+      <c r="B95" s="16"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B96" s="17"/>
+      <c r="B96" s="16"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B97" s="17"/>
+      <c r="B97" s="16"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B98" s="17"/>
+      <c r="B98" s="16"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B99" s="17"/>
+      <c r="B99" s="16"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B100" s="17"/>
+      <c r="B100" s="16"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="17"/>
+      <c r="B101" s="16"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="17"/>
+      <c r="B102" s="16"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B103" s="17"/>
+      <c r="B103" s="16"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B104" s="17"/>
+      <c r="B104" s="16"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B105" s="17"/>
+      <c r="B105" s="16"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="18"/>
+      <c r="B106" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B108" s="15"/>
+      <c r="B108" s="14"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B109" s="15"/>
+      <c r="B109" s="14"/>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="15"/>
+      <c r="B110" s="14"/>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B111" s="15"/>
+      <c r="B111" s="14"/>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="15"/>
+      <c r="B112" s="14"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B113" s="15"/>
+      <c r="B113" s="14"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B114" s="15"/>
+      <c r="B114" s="14"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B115" s="15"/>
+      <c r="B115" s="14"/>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B116" s="15"/>
+      <c r="B116" s="14"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B117" s="15"/>
+      <c r="B117" s="14"/>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B118" s="15"/>
+      <c r="B118" s="14"/>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B119" s="15"/>
+      <c r="B119" s="14"/>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B120" s="15"/>
+      <c r="B120" s="14"/>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B121" s="15"/>
+      <c r="B121" s="14"/>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B122" s="15"/>
+      <c r="B122" s="14"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B123" s="15"/>
+      <c r="B123" s="14"/>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B124" s="15"/>
+      <c r="B124" s="14"/>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B125" s="15"/>
+      <c r="B125" s="14"/>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B126" s="15"/>
+      <c r="B126" s="14"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B127" s="15"/>
+      <c r="B127" s="14"/>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="15"/>
+      <c r="B128" s="14"/>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="15"/>
+      <c r="B129" s="14"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B130" s="15"/>
+      <c r="B130" s="14"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B131" s="15"/>
+      <c r="B131" s="14"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B132" s="15"/>
+      <c r="B132" s="14"/>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B133" s="15"/>
+      <c r="B133" s="14"/>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B134" s="15"/>
+      <c r="B134" s="14"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B135" s="15"/>
+      <c r="B135" s="14"/>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B136" s="15"/>
+      <c r="B136" s="14"/>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B137" s="15"/>
+      <c r="B137" s="14"/>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="15"/>
+      <c r="B138" s="14"/>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="15"/>
+      <c r="B139" s="14"/>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B140" s="15"/>
+      <c r="B140" s="14"/>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B141" s="15"/>
+      <c r="B141" s="14"/>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B142" s="15"/>
+      <c r="B142" s="14"/>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B143" s="15"/>
+      <c r="B143" s="14"/>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B144" s="15"/>
+      <c r="B144" s="14"/>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B145" s="15"/>
+      <c r="B145" s="14"/>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B146" s="15"/>
+      <c r="B146" s="14"/>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B148" s="19"/>
+      <c r="B148" s="18"/>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B149" s="19"/>
+      <c r="B149" s="18"/>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B150" s="19"/>
+      <c r="B150" s="18"/>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B151" s="19"/>
+      <c r="B151" s="18"/>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B152" s="19"/>
+      <c r="B152" s="18"/>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B153" s="19"/>
+      <c r="B153" s="18"/>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B154" s="19"/>
+      <c r="B154" s="18"/>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B155" s="19"/>
+      <c r="B155" s="18"/>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B156" s="19"/>
+      <c r="B156" s="18"/>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B157" s="19"/>
+      <c r="B157" s="18"/>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B158" s="19"/>
+      <c r="B158" s="18"/>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B160" s="19"/>
+      <c r="B160" s="18"/>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B161" s="19"/>
+      <c r="B161" s="18"/>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B162" s="19"/>
+      <c r="B162" s="18"/>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B163" s="19"/>
+      <c r="B163" s="18"/>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B164" s="19"/>
+      <c r="B164" s="18"/>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B165" s="19"/>
+      <c r="B165" s="18"/>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B166" s="19"/>
+      <c r="B166" s="18"/>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B167" s="19"/>
+      <c r="B167" s="18"/>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B168" s="19"/>
+      <c r="B168" s="18"/>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B169" s="19"/>
+      <c r="B169" s="18"/>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B170" s="19"/>
+      <c r="B170" s="18"/>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B171" s="19"/>
+      <c r="B171" s="18"/>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B173" s="19"/>
+      <c r="B173" s="18"/>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B174" s="19"/>
+      <c r="B174" s="18"/>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B175" s="19"/>
+      <c r="B175" s="18"/>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B176" s="19"/>
+      <c r="B176" s="18"/>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B177" s="19"/>
+      <c r="B177" s="18"/>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B178" s="19"/>
+      <c r="B178" s="18"/>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B179" s="19"/>
+      <c r="B179" s="18"/>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B180" s="19"/>
+      <c r="B180" s="18"/>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B181" s="19"/>
+      <c r="B181" s="18"/>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B182" s="19"/>
+      <c r="B182" s="18"/>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B184" s="19"/>
+      <c r="B184" s="18"/>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B185" s="19"/>
+      <c r="B185" s="18"/>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B186" s="19"/>
+      <c r="B186" s="18"/>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B187" s="19"/>
+      <c r="B187" s="18"/>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B188" s="19"/>
+      <c r="B188" s="18"/>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B189" s="19"/>
+      <c r="B189" s="18"/>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B190" s="19"/>
+      <c r="B190" s="18"/>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B191" s="19"/>
+      <c r="B191" s="18"/>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B192" s="19"/>
+      <c r="B192" s="18"/>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B193" s="19"/>
+      <c r="B193" s="18"/>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B195" s="20"/>
+      <c r="B195" s="19"/>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B196" s="20"/>
+      <c r="B196" s="19"/>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B197" s="20"/>
+      <c r="B197" s="19"/>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B198" s="20"/>
+      <c r="B198" s="19"/>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B199" s="20"/>
+      <c r="B199" s="19"/>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B201" s="19"/>
+      <c r="B201" s="18"/>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B202" s="19"/>
+      <c r="B202" s="18"/>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B203" s="19"/>
+      <c r="B203" s="18"/>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B204" s="19"/>
+      <c r="B204" s="18"/>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B205" s="19"/>
+      <c r="B205" s="18"/>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B206" s="19"/>
+      <c r="B206" s="18"/>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B207" s="19"/>
+      <c r="B207" s="18"/>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B208" s="19"/>
+      <c r="B208" s="18"/>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B209" s="19"/>
+      <c r="B209" s="18"/>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B211" s="17"/>
+      <c r="B211" s="16"/>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B212" s="17"/>
+      <c r="B212" s="16"/>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B213" s="17"/>
+      <c r="B213" s="16"/>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B214" s="17"/>
+      <c r="B214" s="16"/>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B215" s="17"/>
+      <c r="B215" s="16"/>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B216" s="17"/>
+      <c r="B216" s="16"/>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B217" s="18"/>
+      <c r="B217" s="17"/>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B218" s="6"/>
+      <c r="B218" s="5"/>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B219" s="17"/>
+      <c r="B219" s="16"/>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B220" s="18"/>
+      <c r="B220" s="17"/>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B221" s="15"/>
+      <c r="B221" s="14"/>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B222" s="15"/>
+      <c r="B222" s="14"/>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B223" s="15"/>
+      <c r="B223" s="14"/>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B224" s="15"/>
+      <c r="B224" s="14"/>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B226" s="15"/>
+      <c r="B226" s="14"/>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B227" s="15"/>
+      <c r="B227" s="14"/>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B228" s="19"/>
+      <c r="B228" s="18"/>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B229" s="19"/>
+      <c r="B229" s="18"/>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B230" s="19"/>
+      <c r="B230" s="18"/>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B231" s="19"/>
+      <c r="B231" s="18"/>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B232" s="19"/>
+      <c r="B232" s="18"/>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B233" s="19"/>
+      <c r="B233" s="18"/>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B234" s="19"/>
+      <c r="B234" s="18"/>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B236" s="17"/>
+      <c r="B236" s="16"/>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B237" s="17"/>
+      <c r="B237" s="16"/>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B238" s="17"/>
+      <c r="B238" s="16"/>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B239" s="17"/>
+      <c r="B239" s="16"/>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B240" s="17"/>
+      <c r="B240" s="16"/>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B241" s="17"/>
+      <c r="B241" s="16"/>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B242" s="18"/>
+      <c r="B242" s="17"/>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B243" s="6"/>
+      <c r="B243" s="5"/>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B244" s="17"/>
+      <c r="B244" s="16"/>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B245" s="18"/>
+      <c r="B245" s="17"/>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B246" s="19"/>
+      <c r="B246" s="18"/>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B247" s="19"/>
+      <c r="B247" s="18"/>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B248" s="19"/>
+      <c r="B248" s="18"/>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B249" s="19"/>
+      <c r="B249" s="18"/>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B250" s="19"/>
+      <c r="B250" s="18"/>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B251" s="19"/>
+      <c r="B251" s="18"/>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B252" s="19"/>
+      <c r="B252" s="18"/>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B253" s="19"/>
+      <c r="B253" s="18"/>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B254" s="19"/>
+      <c r="B254" s="18"/>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B255" s="19"/>
+      <c r="B255" s="18"/>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B256" s="19"/>
+      <c r="B256" s="18"/>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B257" s="19"/>
+      <c r="B257" s="18"/>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B258" s="19"/>
+      <c r="B258" s="18"/>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B259" s="19"/>
+      <c r="B259" s="18"/>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B260" s="19"/>
+      <c r="B260" s="18"/>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B261" s="19"/>
+      <c r="B261" s="18"/>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B262" s="19"/>
+      <c r="B262" s="18"/>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B263" s="19"/>
+      <c r="B263" s="18"/>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B264" s="19"/>
+      <c r="B264" s="18"/>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B265" s="19"/>
+      <c r="B265" s="18"/>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B266" s="19"/>
+      <c r="B266" s="18"/>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B267" s="19"/>
+      <c r="B267" s="18"/>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B268" s="19"/>
+      <c r="B268" s="18"/>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B269" s="19"/>
+      <c r="B269" s="18"/>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B270" s="19"/>
+      <c r="B270" s="18"/>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B271" s="19"/>
+      <c r="B271" s="18"/>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B272" s="19"/>
+      <c r="B272" s="18"/>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B273" s="19"/>
+      <c r="B273" s="18"/>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B274" s="19"/>
+      <c r="B274" s="18"/>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B275" s="19"/>
+      <c r="B275" s="18"/>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B276" s="19"/>
+      <c r="B276" s="18"/>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B277" s="19"/>
+      <c r="B277" s="18"/>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B278" s="19"/>
+      <c r="B278" s="18"/>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B279" s="19"/>
+      <c r="B279" s="18"/>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B280" s="19"/>
+      <c r="B280" s="18"/>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B281" s="19"/>
+      <c r="B281" s="18"/>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B282" s="21"/>
+      <c r="B282" s="20"/>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B284" s="19"/>
+      <c r="B284" s="18"/>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B285" s="19"/>
+      <c r="B285" s="18"/>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B286" s="19"/>
+      <c r="B286" s="18"/>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B287" s="19"/>
+      <c r="B287" s="18"/>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B288" s="19"/>
+      <c r="B288" s="18"/>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B289" s="19"/>
+      <c r="B289" s="18"/>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B290" s="19"/>
+      <c r="B290" s="18"/>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B291" s="19"/>
+      <c r="B291" s="18"/>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B292" s="19"/>
+      <c r="B292" s="18"/>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B293" s="19"/>
+      <c r="B293" s="18"/>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B294" s="19"/>
+      <c r="B294" s="18"/>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B295" s="19"/>
+      <c r="B295" s="18"/>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B296" s="19"/>
+      <c r="B296" s="18"/>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B297" s="19"/>
+      <c r="B297" s="18"/>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B298" s="19"/>
+      <c r="B298" s="18"/>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B299" s="19"/>
+      <c r="B299" s="18"/>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B300" s="19"/>
+      <c r="B300" s="18"/>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B301" s="19"/>
+      <c r="B301" s="18"/>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B302" s="19"/>
+      <c r="B302" s="18"/>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B303" s="19"/>
+      <c r="B303" s="18"/>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B304" s="19"/>
+      <c r="B304" s="18"/>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B305" s="19"/>
+      <c r="B305" s="18"/>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B306" s="19"/>
+      <c r="B306" s="18"/>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B307" s="19"/>
+      <c r="B307" s="18"/>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B308" s="19"/>
+      <c r="B308" s="18"/>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B309" s="19"/>
+      <c r="B309" s="18"/>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B310" s="19"/>
+      <c r="B310" s="18"/>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B311" s="19"/>
+      <c r="B311" s="18"/>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B312" s="19"/>
+      <c r="B312" s="18"/>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B313" s="19"/>
+      <c r="B313" s="18"/>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B314" s="19"/>
+      <c r="B314" s="18"/>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B315" s="19"/>
+      <c r="B315" s="18"/>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B316" s="19"/>
+      <c r="B316" s="18"/>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B317" s="19"/>
+      <c r="B317" s="18"/>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B318" s="19"/>
+      <c r="B318" s="18"/>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B319" s="19"/>
+      <c r="B319" s="18"/>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B320" s="19"/>
+      <c r="B320" s="18"/>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B322" s="17"/>
+      <c r="B322" s="16"/>
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B323" s="17"/>
+      <c r="B323" s="16"/>
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B324" s="17"/>
+      <c r="B324" s="16"/>
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B325" s="17"/>
+      <c r="B325" s="16"/>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B326" s="17"/>
+      <c r="B326" s="16"/>
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B327" s="17"/>
+      <c r="B327" s="16"/>
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B328" s="18"/>
+      <c r="B328" s="17"/>
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B329" s="6"/>
+      <c r="B329" s="5"/>
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B330" s="17"/>
+      <c r="B330" s="16"/>
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B331" s="18"/>
+      <c r="B331" s="17"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D91"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="43.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.58"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="25" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="25" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D44" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="25" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D45" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="25" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="25" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="25" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="25" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="25" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="25" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D53" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="25" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D54" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="25" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="25" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D56" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="25" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D57" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D58" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="25" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D59" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="25" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D60" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C61" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D61" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C62" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D62" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="25" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D63" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="25" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C64" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D64" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="25" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D65" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="25" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C66" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D66" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="25" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D67" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="25" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C68" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D68" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="25" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D69" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="25" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C70" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D70" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D71" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="25" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C72" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D72" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="25" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D73" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="25" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C74" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D74" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="25" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D75" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="25" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C76" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D76" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="25" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D77" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="25" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C78" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D78" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="25" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D79" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="25" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D80" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D81" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="25" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C82" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D82" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="25" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D83" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="25" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C84" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D84" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="25" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C85" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D85" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="25" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C86" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D86" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="25" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C87" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D87" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="25" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C88" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D88" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="25" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="C89" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D89" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="25" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C90" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D90" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="25" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C91" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D91" s="25" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>